<commit_message>
Correction : fins de ligne CRLF dans le module VBA
Le module etait livre avec des fins de ligne Unix (LF seuls). L'editeur VBA
de Windows attend des CRLF : avec des LF seuls il lit tout le module comme
une ligne unique et l'import echoue.

- build_module.py produit et controle les deux formes livrables du module :
  VP_Candidatures.bas (avec Attribute VB_Name, pour Fichier > Importer) et
  VP_Candidatures_a_coller.txt (sans Attribute, pour Insertion > Module puis
  copier-coller, qui contourne toute question de fins de ligne)
- verifier.py controle desormais le format du module : CRLF, Windows-1252,
  presence ou absence de la ligne Attribute, longueur de ligne (max 1023)
  et nombre de continuations (max 24)
- notice du classeur : etape 4 bis (copier-coller) et deux entrees de
  depannage supplementaires

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WfEDN7CVmf69apmMQyJ57N
</commit_message>
<xml_diff>
--- a/outils/gestion-candidatures/Gestion_Candidatures_VP.xlsx
+++ b/outils/gestion-candidatures/Gestion_Candidatures_VP.xlsx
@@ -1991,7 +1991,7 @@
         </is>
       </c>
       <c r="G5" s="33" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="H5" s="30" t="inlineStr">
         <is>
@@ -2032,7 +2032,7 @@
         </is>
       </c>
       <c r="P5" s="33" t="n">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="Q5" s="36" t="n">
         <v>42000</v>
@@ -2046,7 +2046,7 @@
         <v>4</v>
       </c>
       <c r="T5" s="38" t="n">
-        <v>46285.41666666666</v>
+        <v>46286.41666666666</v>
       </c>
       <c r="U5" s="30" t="inlineStr">
         <is>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="V5" s="30" t="n"/>
       <c r="W5" s="33" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="X5" s="30" t="inlineStr">
         <is>
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="Y5" s="33" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="Z5" s="39">
         <f>IF(OR($A5="",$G5="",$W5=""),"",$W5-$G5)</f>
@@ -3682,7 +3682,7 @@
         <v/>
       </c>
       <c r="E4" s="33" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="F4" s="43" t="n">
         <v>0.4166666666666667</v>
@@ -5503,7 +5503,7 @@
     </row>
     <row r="4">
       <c r="A4" s="70" t="n">
-        <v>46280.67708333334</v>
+        <v>46281.28611111111</v>
       </c>
       <c r="B4" s="71" t="inlineStr">
         <is>
@@ -7187,7 +7187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -7436,7 +7436,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1">
+    <row r="28" ht="39" customHeight="1">
       <c r="B28" s="82" t="inlineStr">
         <is>
           <t>4.  Importer le module</t>
@@ -7444,510 +7444,546 @@
       </c>
       <c r="C28" s="83" t="inlineStr">
         <is>
-          <t>Dans l'éditeur : menu Fichier ▸ Importer un fichier… ▸ sélectionnez VP_Candidatures.bas ▸ Ouvrir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="27" customHeight="1">
+          <t>Dans l'éditeur : menu Fichier ▸ Importer un fichier… (raccourci Ctrl + M) ▸ sélectionnez VP_Candidatures.bas ▸ Ouvrir. Un élément « VP_Candidatures » apparaît sous Modules, à gauche, dans l'arborescence du classeur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="39" customHeight="1">
       <c r="B29" s="82" t="inlineStr">
         <is>
+          <t>4 bis.  Si l'import échoue</t>
+        </is>
+      </c>
+      <c r="C29" s="83" t="inlineStr">
+        <is>
+          <t>Utilisez la variante copier-coller, qui fonctionne dans tous les cas : dans l'éditeur, menu Insertion ▸ Module ; ouvrez VP_Candidatures_a_coller.txt avec le Bloc-notes ; Ctrl + A puis Ctrl + C ; revenez dans la fenêtre blanche de l'éditeur et faites Ctrl + V.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="27" customHeight="1">
+      <c r="B30" s="82" t="inlineStr">
+        <is>
           <t>5.  Lancer l'installation</t>
         </is>
       </c>
-      <c r="C29" s="83" t="inlineStr">
+      <c r="C30" s="83" t="inlineStr">
         <is>
           <t>Toujours dans l'éditeur : menu Exécution ▸ Exécuter Sub/UserForm, choisissez « Installer » ▸ Exécuter. Les boutons apparaissent alors dans l'onglet Accueil et en haut de l'onglet Candidatures.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1">
-      <c r="B30" s="82" t="inlineStr">
+    <row r="31" ht="15" customHeight="1">
+      <c r="B31" s="82" t="inlineStr">
         <is>
           <t>6.  Enregistrer</t>
         </is>
       </c>
-      <c r="C30" s="83" t="inlineStr">
+      <c r="C31" s="83" t="inlineStr">
         <is>
           <t>Revenez dans Excel (Alt + F11) et enregistrez. C'est terminé.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="28" customHeight="1">
-      <c r="B31" s="84" t="inlineStr">
+    <row r="32" ht="28" customHeight="1">
+      <c r="B32" s="84" t="inlineStr">
         <is>
           <t>ℹ   Si un bandeau jaune « Avertissement de sécurité » s'affiche à l'ouverture, cliquez sur « Activer le contenu ». Le classeur est alors considéré comme approuvé sur ce poste.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="B32" s="84" t="inlineStr">
+    <row r="33" ht="16" customHeight="1">
+      <c r="B33" s="84" t="inlineStr">
         <is>
           <t>ℹ   Aucune référence VBA supplémentaire n'est nécessaire : le module dialogue avec Outlook et Word en liaison tardive.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="24" customHeight="1">
-      <c r="B34" s="14" t="inlineStr">
+    <row r="35" ht="24" customHeight="1">
+      <c r="B35" s="14" t="inlineStr">
         <is>
           <t>4.  CE QUE FAIT CHAQUE BOUTON</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1">
-      <c r="B35" s="82" t="inlineStr">
+    <row r="36" ht="15" customHeight="1">
+      <c r="B36" s="82" t="inlineStr">
         <is>
           <t>Nouvelle candidature</t>
         </is>
       </c>
-      <c r="C35" s="83" t="inlineStr">
+      <c r="C36" s="83" t="inlineStr">
         <is>
           <t>Ajoute une ligne, attribue l'identifiant (CAND-année-numéro) et la date du jour.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="27" customHeight="1">
-      <c r="B36" s="82" t="inlineStr">
-        <is>
-          <t>Importer depuis Outlook</t>
-        </is>
-      </c>
-      <c r="C36" s="83" t="inlineStr">
-        <is>
-          <t>Parcourt le dossier Outlook indiqué dans Paramètres, crée une ligne par message non lu, enregistre les pièces jointes dans le dossier du candidat et marque le message comme lu.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="27" customHeight="1">
       <c r="B37" s="82" t="inlineStr">
         <is>
+          <t>Importer depuis Outlook</t>
+        </is>
+      </c>
+      <c r="C37" s="83" t="inlineStr">
+        <is>
+          <t>Parcourt le dossier Outlook indiqué dans Paramètres, crée une ligne par message non lu, enregistre les pièces jointes dans le dossier du candidat et marque le message comme lu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="27" customHeight="1">
+      <c r="B38" s="82" t="inlineStr">
+        <is>
           <t>Accusé de réception</t>
         </is>
       </c>
-      <c r="C37" s="83" t="inlineStr">
+      <c r="C38" s="83" t="inlineStr">
         <is>
           <t>Prépare l'e-mail d'accusé de réception, passe le statut à « 2-Accusé de réception » et met à jour la date de dernier contact.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1">
-      <c r="B38" s="82" t="inlineStr">
+    <row r="39" ht="15" customHeight="1">
+      <c r="B39" s="82" t="inlineStr">
         <is>
           <t>Demander des pièces</t>
         </is>
       </c>
-      <c r="C38" s="83" t="inlineStr">
+      <c r="C39" s="83" t="inlineStr">
         <is>
           <t>Envoie la demande de pièces complémentaires et programme une relance.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="27" customHeight="1">
-      <c r="B39" s="82" t="inlineStr">
+    <row r="40" ht="27" customHeight="1">
+      <c r="B40" s="82" t="inlineStr">
         <is>
           <t>Planifier un entretien</t>
         </is>
       </c>
-      <c r="C39" s="83" t="inlineStr">
+      <c r="C40" s="83" t="inlineStr">
         <is>
           <t>Demande la date, l'heure et les modalités ; crée le rendez-vous Outlook avec invitation au candidat, ajoute la ligne dans l'onglet Entretiens et envoie la convocation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="15" customHeight="1">
-      <c r="B40" s="82" t="inlineStr">
-        <is>
-          <t>Mettre en vivier</t>
-        </is>
-      </c>
-      <c r="C40" s="83" t="inlineStr">
-        <is>
-          <t>Envoie le message de mise en vivier et bascule le statut correspondant.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="B41" s="82" t="inlineStr">
         <is>
-          <t>Réponse négative</t>
+          <t>Mettre en vivier</t>
         </is>
       </c>
       <c r="C41" s="83" t="inlineStr">
         <is>
-          <t>Envoie la réponse négative après confirmation, enregistre le motif et clôture le dossier.</t>
+          <t>Envoie le message de mise en vivier et bascule le statut correspondant.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="B42" s="82" t="inlineStr">
         <is>
-          <t>Proposition / suite favorable</t>
+          <t>Réponse négative</t>
         </is>
       </c>
       <c r="C42" s="83" t="inlineStr">
         <is>
-          <t>Envoie le message de suite favorable et passe le statut à « 7-Proposition envoyée ».</t>
+          <t>Envoie la réponse négative après confirmation, enregistre le motif et clôture le dossier.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="B43" s="82" t="inlineStr">
         <is>
-          <t>Envoi groupé</t>
+          <t>Proposition / suite favorable</t>
         </is>
       </c>
       <c r="C43" s="83" t="inlineStr">
         <is>
-          <t>Applique le même modèle d'e-mail à toutes les lignes sélectionnées (utile quand un poste est pourvu).</t>
+          <t>Envoie le message de suite favorable et passe le statut à « 7-Proposition envoyée ».</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="B44" s="82" t="inlineStr">
         <is>
-          <t>Fiche candidat (Word)</t>
+          <t>Envoi groupé</t>
         </is>
       </c>
       <c r="C44" s="83" t="inlineStr">
         <is>
-          <t>Génère la fiche de synthèse et la grille d'entretien dans le dossier du candidat.</t>
+          <t>Applique le même modèle d'e-mail à toutes les lignes sélectionnées (utile quand un poste est pourvu).</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="B45" s="82" t="inlineStr">
         <is>
-          <t>Courrier de convocation</t>
+          <t>Fiche candidat (Word)</t>
         </is>
       </c>
       <c r="C45" s="83" t="inlineStr">
         <is>
-          <t>Génère la convocation en courrier Word, prête à être signée.</t>
+          <t>Génère la fiche de synthèse et la grille d'entretien dans le dossier du candidat.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="B46" s="82" t="inlineStr">
         <is>
-          <t>Lettre de refus</t>
+          <t>Courrier de convocation</t>
         </is>
       </c>
       <c r="C46" s="83" t="inlineStr">
         <is>
-          <t>Génère la lettre de refus sur papier à en-tête.</t>
+          <t>Génère la convocation en courrier Word, prête à être signée.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="B47" s="82" t="inlineStr">
         <is>
-          <t>Convention / promesse</t>
+          <t>Lettre de refus</t>
         </is>
       </c>
       <c r="C47" s="83" t="inlineStr">
         <is>
-          <t>Génère la convention de stage ou la promesse d'embauche à partir du modèle.</t>
+          <t>Génère la lettre de refus sur papier à en-tête.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="B48" s="82" t="inlineStr">
         <is>
-          <t>Dossier du candidat</t>
+          <t>Convention / promesse</t>
         </is>
       </c>
       <c r="C48" s="83" t="inlineStr">
         <is>
-          <t>Crée le dossier du candidat s'il n'existe pas et l'ouvre dans l'Explorateur.</t>
+          <t>Génère la convention de stage ou la promesse d'embauche à partir du modèle.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="B49" s="82" t="inlineStr">
         <is>
-          <t>Relances à faire</t>
+          <t>Dossier du candidat</t>
         </is>
       </c>
       <c r="C49" s="83" t="inlineStr">
         <is>
-          <t>Liste les dossiers en retard et crée une tâche Outlook pour chacun.</t>
+          <t>Crée le dossier du candidat s'il n'existe pas et l'ouvre dans l'Explorateur.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="B50" s="82" t="inlineStr">
         <is>
-          <t>Purge RGPD</t>
+          <t>Relances à faire</t>
         </is>
       </c>
       <c r="C50" s="83" t="inlineStr">
         <is>
-          <t>Recense les candidatures dont la durée de conservation est dépassée et propose leur anonymisation.</t>
+          <t>Liste les dossiers en retard et crée une tâche Outlook pour chacun.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="B51" s="82" t="inlineStr">
         <is>
-          <t>Actualiser les listes</t>
+          <t>Purge RGPD</t>
         </is>
       </c>
       <c r="C51" s="83" t="inlineStr">
         <is>
-          <t>Étend les menus déroulants après l'ajout de valeurs dans l'onglet Paramètres.</t>
+          <t>Recense les candidatures dont la durée de conservation est dépassée et propose leur anonymisation.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="B52" s="82" t="inlineStr">
         <is>
+          <t>Actualiser les listes</t>
+        </is>
+      </c>
+      <c r="C52" s="83" t="inlineStr">
+        <is>
+          <t>Étend les menus déroulants après l'ajout de valeurs dans l'onglet Paramètres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="15" customHeight="1">
+      <c r="B53" s="82" t="inlineStr">
+        <is>
           <t>Supprimer les exemples</t>
         </is>
       </c>
-      <c r="C52" s="83" t="inlineStr">
+      <c r="C53" s="83" t="inlineStr">
         <is>
           <t>Supprime les lignes de démonstration (EXEMPLE-…) des onglets Candidatures et Entretiens.</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="24" customHeight="1">
-      <c r="B54" s="14" t="inlineStr">
+    <row r="55" ht="24" customHeight="1">
+      <c r="B55" s="14" t="inlineStr">
         <is>
           <t>5.  LE CIRCUIT TYPE D'UNE CANDIDATURE</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="15" customHeight="1">
-      <c r="B55" s="82" t="inlineStr">
-        <is>
-          <t>Réception</t>
-        </is>
-      </c>
-      <c r="C55" s="83" t="inlineStr">
-        <is>
-          <t>Import Outlook ou saisie manuelle ▸ statut 1-Reçue.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="B56" s="82" t="inlineStr">
         <is>
-          <t>Sous 7 jours</t>
+          <t>Réception</t>
         </is>
       </c>
       <c r="C56" s="83" t="inlineStr">
         <is>
-          <t>Accusé de réception ▸ statut 2. Au-delà, la colonne Alerte affiche « À traiter ».</t>
+          <t>Import Outlook ou saisie manuelle ▸ statut 1-Reçue.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="B57" s="82" t="inlineStr">
         <is>
-          <t>Examen</t>
+          <t>Sous 7 jours</t>
         </is>
       </c>
       <c r="C57" s="83" t="inlineStr">
         <is>
-          <t>Statut 3-En cours d'examen, attribution d'un responsable et d'une note sur 5.</t>
+          <t>Accusé de réception ▸ statut 2. Au-delà, la colonne Alerte affiche « À traiter ».</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="B58" s="82" t="inlineStr">
         <is>
-          <t>Entretien</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="C58" s="83" t="inlineStr">
         <is>
-          <t>Planification ▸ statut 4, puis compte rendu dans l'onglet Entretiens ▸ statut 5.</t>
+          <t>Statut 3-En cours d'examen, attribution d'un responsable et d'une note sur 5.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="B59" s="82" t="inlineStr">
         <is>
-          <t>Décision</t>
+          <t>Entretien</t>
         </is>
       </c>
       <c r="C59" s="83" t="inlineStr">
         <is>
-          <t>Proposition (7) et recrutement (8), vivier (6), ou réponse négative (9).</t>
+          <t>Planification ▸ statut 4, puis compte rendu dans l'onglet Entretiens ▸ statut 5.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="B60" s="82" t="inlineStr">
         <is>
+          <t>Décision</t>
+        </is>
+      </c>
+      <c r="C60" s="83" t="inlineStr">
+        <is>
+          <t>Proposition (7) et recrutement (8), vivier (6), ou réponse négative (9).</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="15" customHeight="1">
+      <c r="B61" s="82" t="inlineStr">
+        <is>
           <t>Après décision</t>
         </is>
       </c>
-      <c r="C60" s="83" t="inlineStr">
+      <c r="C61" s="83" t="inlineStr">
         <is>
           <t>La ligne passe en gris. La date de purge RGPD est calculée automatiquement.</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="24" customHeight="1">
-      <c r="B62" s="14" t="inlineStr">
+    <row r="63" ht="24" customHeight="1">
+      <c r="B63" s="14" t="inlineStr">
         <is>
           <t>6.  PROTECTION DES DONNÉES (RGPD)</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="16" customHeight="1">
-      <c r="B63" s="84" t="inlineStr">
+    <row r="64" ht="16" customHeight="1">
+      <c r="B64" s="84" t="inlineStr">
         <is>
           <t>ℹ   Un fichier de candidatures est un traitement de données personnelles : il doit figurer au registre du cabinet.</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="27" customHeight="1">
-      <c r="B64" s="82" t="inlineStr">
+    <row r="65" ht="27" customHeight="1">
+      <c r="B65" s="82" t="inlineStr">
         <is>
           <t>Conservation</t>
         </is>
       </c>
-      <c r="C64" s="83" t="inlineStr">
+      <c r="C65" s="83" t="inlineStr">
         <is>
           <t>Par défaut 2 ans à compter du dernier contact, conformément à la recommandation de la CNIL. Le délai est modifiable dans Paramètres ; la colonne « Purge RGPD le » se recalcule seule.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="15" customHeight="1">
-      <c r="B65" s="82" t="inlineStr">
-        <is>
-          <t>Information</t>
-        </is>
-      </c>
-      <c r="C65" s="83" t="inlineStr">
-        <is>
-          <t>Les modèles d'e-mails comportent la mention d'information et le rappel des droits du candidat.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="B66" s="82" t="inlineStr">
         <is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="C66" s="83" t="inlineStr">
+        <is>
+          <t>Les modèles d'e-mails comportent la mention d'information et le rappel des droits du candidat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="15" customHeight="1">
+      <c r="B67" s="82" t="inlineStr">
+        <is>
           <t>Vivier</t>
         </is>
       </c>
-      <c r="C66" s="83" t="inlineStr">
+      <c r="C67" s="83" t="inlineStr">
         <is>
           <t>La conservation au-delà du recrutement suppose l'accord du candidat : colonne « Consentement vivier ».</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="27" customHeight="1">
-      <c r="B67" s="82" t="inlineStr">
+    <row r="68" ht="27" customHeight="1">
+      <c r="B68" s="82" t="inlineStr">
         <is>
           <t>Données sensibles</t>
         </is>
       </c>
-      <c r="C67" s="83" t="inlineStr">
+      <c r="C68" s="83" t="inlineStr">
         <is>
           <t>Ne saisissez jamais dans les commentaires d'information sur la santé, l'origine, les opinions politiques, religieuses ou syndicales, ni sur la vie privée du candidat.</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1">
-      <c r="B68" s="82" t="inlineStr">
+    <row r="69" ht="15" customHeight="1">
+      <c r="B69" s="82" t="inlineStr">
         <is>
           <t>Accès</t>
         </is>
       </c>
-      <c r="C68" s="83" t="inlineStr">
+      <c r="C69" s="83" t="inlineStr">
         <is>
           <t>Rangez le classeur dans un dossier à accès restreint et sauvegardez-le régulièrement.</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="24" customHeight="1">
-      <c r="B70" s="14" t="inlineStr">
+    <row r="71" ht="24" customHeight="1">
+      <c r="B71" s="14" t="inlineStr">
         <is>
           <t>7.  DÉPANNAGE</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1">
-      <c r="B71" s="82" t="inlineStr">
-        <is>
-          <t>Les boutons ne réagissent pas</t>
-        </is>
-      </c>
-      <c r="C71" s="83" t="inlineStr">
-        <is>
-          <t>Le fichier a été enregistré en .xlsx, ou les macros sont désactivées : reprenez la section 3.</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="15" customHeight="1">
+    <row r="72" ht="39" customHeight="1">
       <c r="B72" s="82" t="inlineStr">
         <is>
-          <t>« Impossible de lire le fichier »</t>
+          <t>L'import du module échoue</t>
         </is>
       </c>
       <c r="C72" s="83" t="inlineStr">
         <is>
-          <t>Le fichier n'a pas été débloqué : clic droit ▸ Propriétés ▸ Débloquer.</t>
+          <t>Vérifiez le nom exact du fichier : certains navigateurs le téléchargent en VP_Candidatures.bas.txt. Affichez les extensions dans l'Explorateur et renommez-le si besoin. En cas de doute, utilisez directement la variante copier-coller (étape 4 bis).</t>
         </is>
       </c>
     </row>
     <row r="73" ht="27" customHeight="1">
       <c r="B73" s="82" t="inlineStr">
         <is>
-          <t>Outlook ne s'ouvre pas</t>
+          <t>Le module importé est illisible</t>
         </is>
       </c>
       <c r="C73" s="83" t="inlineStr">
         <is>
-          <t>Outlook doit être installé et un profil configuré sur le poste. La version web d'Outlook ne permet pas ce type d'automatisation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="27" customHeight="1">
+          <t>Le fichier a été réenregistré par un éditeur qui a modifié les fins de ligne ou l'encodage. Reprenez le fichier d'origine, ou utilisez la variante copier-coller.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="15" customHeight="1">
       <c r="B74" s="82" t="inlineStr">
         <is>
-          <t>L'e-mail part sans signature</t>
+          <t>Les boutons ne réagissent pas</t>
         </is>
       </c>
       <c r="C74" s="83" t="inlineStr">
         <is>
-          <t>Laissez la cellule « Signature e-mail » vide dans Paramètres : la signature Outlook par défaut est alors conservée.</t>
+          <t>Le fichier a été enregistré en .xlsx, ou les macros sont désactivées : reprenez la section 3.</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="B75" s="82" t="inlineStr">
         <is>
-          <t>Le document Word est vide</t>
+          <t>« Impossible de lire le fichier »</t>
         </is>
       </c>
       <c r="C75" s="83" t="inlineStr">
         <is>
-          <t>Vérifiez le chemin du dossier des modèles dans Paramètres et la présence des fichiers .docx.</t>
+          <t>Le fichier n'a pas été débloqué : clic droit ▸ Propriétés ▸ Débloquer.</t>
         </is>
       </c>
     </row>
     <row r="76" ht="27" customHeight="1">
       <c r="B76" s="82" t="inlineStr">
         <is>
-          <t>Une valeur est refusée</t>
+          <t>Outlook ne s'ouvre pas</t>
         </is>
       </c>
       <c r="C76" s="83" t="inlineStr">
         <is>
-          <t>Elle ne figure pas dans la liste de l'onglet Paramètres : ajoutez-la, puis cliquez sur « Actualiser les listes ».</t>
+          <t>Outlook doit être installé et un profil configuré sur le poste. La version web d'Outlook ne permet pas ce type d'automatisation.</t>
         </is>
       </c>
     </row>
     <row r="77" ht="27" customHeight="1">
       <c r="B77" s="82" t="inlineStr">
         <is>
+          <t>L'e-mail part sans signature</t>
+        </is>
+      </c>
+      <c r="C77" s="83" t="inlineStr">
+        <is>
+          <t>Laissez la cellule « Signature e-mail » vide dans Paramètres : la signature Outlook par défaut est alors conservée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="15" customHeight="1">
+      <c r="B78" s="82" t="inlineStr">
+        <is>
+          <t>Le document Word est vide</t>
+        </is>
+      </c>
+      <c r="C78" s="83" t="inlineStr">
+        <is>
+          <t>Vérifiez le chemin du dossier des modèles dans Paramètres et la présence des fichiers .docx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="27" customHeight="1">
+      <c r="B79" s="82" t="inlineStr">
+        <is>
+          <t>Une valeur est refusée</t>
+        </is>
+      </c>
+      <c r="C79" s="83" t="inlineStr">
+        <is>
+          <t>Elle ne figure pas dans la liste de l'onglet Paramètres : ajoutez-la, puis cliquez sur « Actualiser les listes ».</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="27" customHeight="1">
+      <c r="B80" s="82" t="inlineStr">
+        <is>
           <t>Le classeur devient lent</t>
         </is>
       </c>
-      <c r="C77" s="83" t="inlineStr">
+      <c r="C80" s="83" t="inlineStr">
         <is>
           <t>Supprimez les lignes vides sous le tableau et archivez les candidatures closes de plus de deux ans (bouton Purge RGPD).</t>
         </is>
@@ -7955,19 +7991,19 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B55:C55"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B64:C64"/>
     <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="B33:C33"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B34:C34"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B31:C31"/>
     <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="B35:C35"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Notice : lancement de l'installation independant de la version
Le menu Execution de l'editeur VBA affiche selon les versions
"Executer la macro" ou "Executer Sub/UserForm". La notice ne citait que
le second libelle.

L'etape 5 passe desormais par Excel (Alt+F8 > Installer > Executer), qui
ne depend d'aucun libelle, la variante F5 depuis l'editeur etant donnee
en complement. Une entree de depannage est ajoutee.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WfEDN7CVmf69apmMQyJ57N
</commit_message>
<xml_diff>
--- a/outils/gestion-candidatures/Gestion_Candidatures_VP.xlsx
+++ b/outils/gestion-candidatures/Gestion_Candidatures_VP.xlsx
@@ -5503,7 +5503,7 @@
     </row>
     <row r="4">
       <c r="A4" s="70" t="n">
-        <v>46281.28611111111</v>
+        <v>46281.29166666666</v>
       </c>
       <c r="B4" s="71" t="inlineStr">
         <is>
@@ -7187,7 +7187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -7460,7 +7460,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="27" customHeight="1">
+    <row r="30" ht="39" customHeight="1">
       <c r="B30" s="82" t="inlineStr">
         <is>
           <t>5.  Lancer l'installation</t>
@@ -7468,542 +7468,562 @@
       </c>
       <c r="C30" s="83" t="inlineStr">
         <is>
-          <t>Toujours dans l'éditeur : menu Exécution ▸ Exécuter Sub/UserForm, choisissez « Installer » ▸ Exécuter. Les boutons apparaissent alors dans l'onglet Accueil et en haut de l'onglet Candidatures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="15" customHeight="1">
-      <c r="B31" s="82" t="inlineStr">
+          <t>Revenez dans Excel (Alt + F11) puis appuyez sur Alt + F8 : choisissez « Installer » dans la liste des macros et cliquez sur Exécuter. Les boutons apparaissent alors dans l'onglet Accueil et en haut de l'onglet Candidatures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="40" customHeight="1">
+      <c r="B31" s="84" t="inlineStr">
+        <is>
+          <t>ℹ   Variante depuis l'éditeur : cliquez dans le corps de la procédure Installer, puis appuyez sur F5. Le libellé du menu Exécution varie selon les versions — « Exécuter la macro » ou « Exécuter Sub/UserForm » — mais il s'agit de la même commande, et c'est la position du curseur qui détermine la procédure lancée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="B32" s="82" t="inlineStr">
         <is>
           <t>6.  Enregistrer</t>
         </is>
       </c>
-      <c r="C31" s="83" t="inlineStr">
+      <c r="C32" s="83" t="inlineStr">
         <is>
           <t>Revenez dans Excel (Alt + F11) et enregistrez. C'est terminé.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="B32" s="84" t="inlineStr">
+    <row r="33" ht="28" customHeight="1">
+      <c r="B33" s="84" t="inlineStr">
         <is>
           <t>ℹ   Si un bandeau jaune « Avertissement de sécurité » s'affiche à l'ouverture, cliquez sur « Activer le contenu ». Le classeur est alors considéré comme approuvé sur ce poste.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="B33" s="84" t="inlineStr">
+    <row r="34" ht="16" customHeight="1">
+      <c r="B34" s="84" t="inlineStr">
         <is>
           <t>ℹ   Aucune référence VBA supplémentaire n'est nécessaire : le module dialogue avec Outlook et Word en liaison tardive.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="24" customHeight="1">
-      <c r="B35" s="14" t="inlineStr">
+    <row r="36" ht="24" customHeight="1">
+      <c r="B36" s="14" t="inlineStr">
         <is>
           <t>4.  CE QUE FAIT CHAQUE BOUTON</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="15" customHeight="1">
-      <c r="B36" s="82" t="inlineStr">
+    <row r="37" ht="15" customHeight="1">
+      <c r="B37" s="82" t="inlineStr">
         <is>
           <t>Nouvelle candidature</t>
         </is>
       </c>
-      <c r="C36" s="83" t="inlineStr">
+      <c r="C37" s="83" t="inlineStr">
         <is>
           <t>Ajoute une ligne, attribue l'identifiant (CAND-année-numéro) et la date du jour.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="27" customHeight="1">
-      <c r="B37" s="82" t="inlineStr">
-        <is>
-          <t>Importer depuis Outlook</t>
-        </is>
-      </c>
-      <c r="C37" s="83" t="inlineStr">
-        <is>
-          <t>Parcourt le dossier Outlook indiqué dans Paramètres, crée une ligne par message non lu, enregistre les pièces jointes dans le dossier du candidat et marque le message comme lu.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="27" customHeight="1">
       <c r="B38" s="82" t="inlineStr">
         <is>
+          <t>Importer depuis Outlook</t>
+        </is>
+      </c>
+      <c r="C38" s="83" t="inlineStr">
+        <is>
+          <t>Parcourt le dossier Outlook indiqué dans Paramètres, crée une ligne par message non lu, enregistre les pièces jointes dans le dossier du candidat et marque le message comme lu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="27" customHeight="1">
+      <c r="B39" s="82" t="inlineStr">
+        <is>
           <t>Accusé de réception</t>
         </is>
       </c>
-      <c r="C38" s="83" t="inlineStr">
+      <c r="C39" s="83" t="inlineStr">
         <is>
           <t>Prépare l'e-mail d'accusé de réception, passe le statut à « 2-Accusé de réception » et met à jour la date de dernier contact.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="15" customHeight="1">
-      <c r="B39" s="82" t="inlineStr">
+    <row r="40" ht="15" customHeight="1">
+      <c r="B40" s="82" t="inlineStr">
         <is>
           <t>Demander des pièces</t>
         </is>
       </c>
-      <c r="C39" s="83" t="inlineStr">
+      <c r="C40" s="83" t="inlineStr">
         <is>
           <t>Envoie la demande de pièces complémentaires et programme une relance.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="27" customHeight="1">
-      <c r="B40" s="82" t="inlineStr">
+    <row r="41" ht="27" customHeight="1">
+      <c r="B41" s="82" t="inlineStr">
         <is>
           <t>Planifier un entretien</t>
         </is>
       </c>
-      <c r="C40" s="83" t="inlineStr">
+      <c r="C41" s="83" t="inlineStr">
         <is>
           <t>Demande la date, l'heure et les modalités ; crée le rendez-vous Outlook avec invitation au candidat, ajoute la ligne dans l'onglet Entretiens et envoie la convocation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="15" customHeight="1">
-      <c r="B41" s="82" t="inlineStr">
-        <is>
-          <t>Mettre en vivier</t>
-        </is>
-      </c>
-      <c r="C41" s="83" t="inlineStr">
-        <is>
-          <t>Envoie le message de mise en vivier et bascule le statut correspondant.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="B42" s="82" t="inlineStr">
         <is>
-          <t>Réponse négative</t>
+          <t>Mettre en vivier</t>
         </is>
       </c>
       <c r="C42" s="83" t="inlineStr">
         <is>
-          <t>Envoie la réponse négative après confirmation, enregistre le motif et clôture le dossier.</t>
+          <t>Envoie le message de mise en vivier et bascule le statut correspondant.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="B43" s="82" t="inlineStr">
         <is>
-          <t>Proposition / suite favorable</t>
+          <t>Réponse négative</t>
         </is>
       </c>
       <c r="C43" s="83" t="inlineStr">
         <is>
-          <t>Envoie le message de suite favorable et passe le statut à « 7-Proposition envoyée ».</t>
+          <t>Envoie la réponse négative après confirmation, enregistre le motif et clôture le dossier.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="B44" s="82" t="inlineStr">
         <is>
-          <t>Envoi groupé</t>
+          <t>Proposition / suite favorable</t>
         </is>
       </c>
       <c r="C44" s="83" t="inlineStr">
         <is>
-          <t>Applique le même modèle d'e-mail à toutes les lignes sélectionnées (utile quand un poste est pourvu).</t>
+          <t>Envoie le message de suite favorable et passe le statut à « 7-Proposition envoyée ».</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="B45" s="82" t="inlineStr">
         <is>
-          <t>Fiche candidat (Word)</t>
+          <t>Envoi groupé</t>
         </is>
       </c>
       <c r="C45" s="83" t="inlineStr">
         <is>
-          <t>Génère la fiche de synthèse et la grille d'entretien dans le dossier du candidat.</t>
+          <t>Applique le même modèle d'e-mail à toutes les lignes sélectionnées (utile quand un poste est pourvu).</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="B46" s="82" t="inlineStr">
         <is>
-          <t>Courrier de convocation</t>
+          <t>Fiche candidat (Word)</t>
         </is>
       </c>
       <c r="C46" s="83" t="inlineStr">
         <is>
-          <t>Génère la convocation en courrier Word, prête à être signée.</t>
+          <t>Génère la fiche de synthèse et la grille d'entretien dans le dossier du candidat.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="B47" s="82" t="inlineStr">
         <is>
-          <t>Lettre de refus</t>
+          <t>Courrier de convocation</t>
         </is>
       </c>
       <c r="C47" s="83" t="inlineStr">
         <is>
-          <t>Génère la lettre de refus sur papier à en-tête.</t>
+          <t>Génère la convocation en courrier Word, prête à être signée.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="B48" s="82" t="inlineStr">
         <is>
-          <t>Convention / promesse</t>
+          <t>Lettre de refus</t>
         </is>
       </c>
       <c r="C48" s="83" t="inlineStr">
         <is>
-          <t>Génère la convention de stage ou la promesse d'embauche à partir du modèle.</t>
+          <t>Génère la lettre de refus sur papier à en-tête.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="B49" s="82" t="inlineStr">
         <is>
-          <t>Dossier du candidat</t>
+          <t>Convention / promesse</t>
         </is>
       </c>
       <c r="C49" s="83" t="inlineStr">
         <is>
-          <t>Crée le dossier du candidat s'il n'existe pas et l'ouvre dans l'Explorateur.</t>
+          <t>Génère la convention de stage ou la promesse d'embauche à partir du modèle.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="B50" s="82" t="inlineStr">
         <is>
-          <t>Relances à faire</t>
+          <t>Dossier du candidat</t>
         </is>
       </c>
       <c r="C50" s="83" t="inlineStr">
         <is>
-          <t>Liste les dossiers en retard et crée une tâche Outlook pour chacun.</t>
+          <t>Crée le dossier du candidat s'il n'existe pas et l'ouvre dans l'Explorateur.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="B51" s="82" t="inlineStr">
         <is>
-          <t>Purge RGPD</t>
+          <t>Relances à faire</t>
         </is>
       </c>
       <c r="C51" s="83" t="inlineStr">
         <is>
-          <t>Recense les candidatures dont la durée de conservation est dépassée et propose leur anonymisation.</t>
+          <t>Liste les dossiers en retard et crée une tâche Outlook pour chacun.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="B52" s="82" t="inlineStr">
         <is>
-          <t>Actualiser les listes</t>
+          <t>Purge RGPD</t>
         </is>
       </c>
       <c r="C52" s="83" t="inlineStr">
         <is>
-          <t>Étend les menus déroulants après l'ajout de valeurs dans l'onglet Paramètres.</t>
+          <t>Recense les candidatures dont la durée de conservation est dépassée et propose leur anonymisation.</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="B53" s="82" t="inlineStr">
         <is>
+          <t>Actualiser les listes</t>
+        </is>
+      </c>
+      <c r="C53" s="83" t="inlineStr">
+        <is>
+          <t>Étend les menus déroulants après l'ajout de valeurs dans l'onglet Paramètres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="15" customHeight="1">
+      <c r="B54" s="82" t="inlineStr">
+        <is>
           <t>Supprimer les exemples</t>
         </is>
       </c>
-      <c r="C53" s="83" t="inlineStr">
+      <c r="C54" s="83" t="inlineStr">
         <is>
           <t>Supprime les lignes de démonstration (EXEMPLE-…) des onglets Candidatures et Entretiens.</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="24" customHeight="1">
-      <c r="B55" s="14" t="inlineStr">
+    <row r="56" ht="24" customHeight="1">
+      <c r="B56" s="14" t="inlineStr">
         <is>
           <t>5.  LE CIRCUIT TYPE D'UNE CANDIDATURE</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="15" customHeight="1">
-      <c r="B56" s="82" t="inlineStr">
-        <is>
-          <t>Réception</t>
-        </is>
-      </c>
-      <c r="C56" s="83" t="inlineStr">
-        <is>
-          <t>Import Outlook ou saisie manuelle ▸ statut 1-Reçue.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="B57" s="82" t="inlineStr">
         <is>
-          <t>Sous 7 jours</t>
+          <t>Réception</t>
         </is>
       </c>
       <c r="C57" s="83" t="inlineStr">
         <is>
-          <t>Accusé de réception ▸ statut 2. Au-delà, la colonne Alerte affiche « À traiter ».</t>
+          <t>Import Outlook ou saisie manuelle ▸ statut 1-Reçue.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="B58" s="82" t="inlineStr">
         <is>
-          <t>Examen</t>
+          <t>Sous 7 jours</t>
         </is>
       </c>
       <c r="C58" s="83" t="inlineStr">
         <is>
-          <t>Statut 3-En cours d'examen, attribution d'un responsable et d'une note sur 5.</t>
+          <t>Accusé de réception ▸ statut 2. Au-delà, la colonne Alerte affiche « À traiter ».</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="B59" s="82" t="inlineStr">
         <is>
-          <t>Entretien</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="C59" s="83" t="inlineStr">
         <is>
-          <t>Planification ▸ statut 4, puis compte rendu dans l'onglet Entretiens ▸ statut 5.</t>
+          <t>Statut 3-En cours d'examen, attribution d'un responsable et d'une note sur 5.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="B60" s="82" t="inlineStr">
         <is>
-          <t>Décision</t>
+          <t>Entretien</t>
         </is>
       </c>
       <c r="C60" s="83" t="inlineStr">
         <is>
-          <t>Proposition (7) et recrutement (8), vivier (6), ou réponse négative (9).</t>
+          <t>Planification ▸ statut 4, puis compte rendu dans l'onglet Entretiens ▸ statut 5.</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="B61" s="82" t="inlineStr">
         <is>
+          <t>Décision</t>
+        </is>
+      </c>
+      <c r="C61" s="83" t="inlineStr">
+        <is>
+          <t>Proposition (7) et recrutement (8), vivier (6), ou réponse négative (9).</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="15" customHeight="1">
+      <c r="B62" s="82" t="inlineStr">
+        <is>
           <t>Après décision</t>
         </is>
       </c>
-      <c r="C61" s="83" t="inlineStr">
+      <c r="C62" s="83" t="inlineStr">
         <is>
           <t>La ligne passe en gris. La date de purge RGPD est calculée automatiquement.</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="24" customHeight="1">
-      <c r="B63" s="14" t="inlineStr">
+    <row r="64" ht="24" customHeight="1">
+      <c r="B64" s="14" t="inlineStr">
         <is>
           <t>6.  PROTECTION DES DONNÉES (RGPD)</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="16" customHeight="1">
-      <c r="B64" s="84" t="inlineStr">
+    <row r="65" ht="16" customHeight="1">
+      <c r="B65" s="84" t="inlineStr">
         <is>
           <t>ℹ   Un fichier de candidatures est un traitement de données personnelles : il doit figurer au registre du cabinet.</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="27" customHeight="1">
-      <c r="B65" s="82" t="inlineStr">
+    <row r="66" ht="27" customHeight="1">
+      <c r="B66" s="82" t="inlineStr">
         <is>
           <t>Conservation</t>
         </is>
       </c>
-      <c r="C65" s="83" t="inlineStr">
+      <c r="C66" s="83" t="inlineStr">
         <is>
           <t>Par défaut 2 ans à compter du dernier contact, conformément à la recommandation de la CNIL. Le délai est modifiable dans Paramètres ; la colonne « Purge RGPD le » se recalcule seule.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="15" customHeight="1">
-      <c r="B66" s="82" t="inlineStr">
-        <is>
-          <t>Information</t>
-        </is>
-      </c>
-      <c r="C66" s="83" t="inlineStr">
-        <is>
-          <t>Les modèles d'e-mails comportent la mention d'information et le rappel des droits du candidat.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="B67" s="82" t="inlineStr">
         <is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="C67" s="83" t="inlineStr">
+        <is>
+          <t>Les modèles d'e-mails comportent la mention d'information et le rappel des droits du candidat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="15" customHeight="1">
+      <c r="B68" s="82" t="inlineStr">
+        <is>
           <t>Vivier</t>
         </is>
       </c>
-      <c r="C67" s="83" t="inlineStr">
+      <c r="C68" s="83" t="inlineStr">
         <is>
           <t>La conservation au-delà du recrutement suppose l'accord du candidat : colonne « Consentement vivier ».</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="27" customHeight="1">
-      <c r="B68" s="82" t="inlineStr">
+    <row r="69" ht="27" customHeight="1">
+      <c r="B69" s="82" t="inlineStr">
         <is>
           <t>Données sensibles</t>
         </is>
       </c>
-      <c r="C68" s="83" t="inlineStr">
+      <c r="C69" s="83" t="inlineStr">
         <is>
           <t>Ne saisissez jamais dans les commentaires d'information sur la santé, l'origine, les opinions politiques, religieuses ou syndicales, ni sur la vie privée du candidat.</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="15" customHeight="1">
-      <c r="B69" s="82" t="inlineStr">
+    <row r="70" ht="15" customHeight="1">
+      <c r="B70" s="82" t="inlineStr">
         <is>
           <t>Accès</t>
         </is>
       </c>
-      <c r="C69" s="83" t="inlineStr">
+      <c r="C70" s="83" t="inlineStr">
         <is>
           <t>Rangez le classeur dans un dossier à accès restreint et sauvegardez-le régulièrement.</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="24" customHeight="1">
-      <c r="B71" s="14" t="inlineStr">
+    <row r="72" ht="24" customHeight="1">
+      <c r="B72" s="14" t="inlineStr">
         <is>
           <t>7.  DÉPANNAGE</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="39" customHeight="1">
-      <c r="B72" s="82" t="inlineStr">
+    <row r="73" ht="39" customHeight="1">
+      <c r="B73" s="82" t="inlineStr">
+        <is>
+          <t>Je ne trouve pas la commande d'exécution</t>
+        </is>
+      </c>
+      <c r="C73" s="83" t="inlineStr">
+        <is>
+          <t>Le libellé diffère d'une version à l'autre. Le plus simple est de passer par Excel : Alt + F8, sélectionnez « Installer », puis Exécuter. Si la liste est vide, le module n'a pas été importé dans ce classeur : vérifiez qu'il figure bien sous Modules dans l'arborescence de l'éditeur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="39" customHeight="1">
+      <c r="B74" s="82" t="inlineStr">
         <is>
           <t>L'import du module échoue</t>
         </is>
       </c>
-      <c r="C72" s="83" t="inlineStr">
+      <c r="C74" s="83" t="inlineStr">
         <is>
           <t>Vérifiez le nom exact du fichier : certains navigateurs le téléchargent en VP_Candidatures.bas.txt. Affichez les extensions dans l'Explorateur et renommez-le si besoin. En cas de doute, utilisez directement la variante copier-coller (étape 4 bis).</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="27" customHeight="1">
-      <c r="B73" s="82" t="inlineStr">
+    <row r="75" ht="27" customHeight="1">
+      <c r="B75" s="82" t="inlineStr">
         <is>
           <t>Le module importé est illisible</t>
         </is>
       </c>
-      <c r="C73" s="83" t="inlineStr">
+      <c r="C75" s="83" t="inlineStr">
         <is>
           <t>Le fichier a été réenregistré par un éditeur qui a modifié les fins de ligne ou l'encodage. Reprenez le fichier d'origine, ou utilisez la variante copier-coller.</t>
         </is>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1">
-      <c r="B74" s="82" t="inlineStr">
+    <row r="76" ht="15" customHeight="1">
+      <c r="B76" s="82" t="inlineStr">
         <is>
           <t>Les boutons ne réagissent pas</t>
         </is>
       </c>
-      <c r="C74" s="83" t="inlineStr">
+      <c r="C76" s="83" t="inlineStr">
         <is>
           <t>Le fichier a été enregistré en .xlsx, ou les macros sont désactivées : reprenez la section 3.</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1">
-      <c r="B75" s="82" t="inlineStr">
+    <row r="77" ht="15" customHeight="1">
+      <c r="B77" s="82" t="inlineStr">
         <is>
           <t>« Impossible de lire le fichier »</t>
         </is>
       </c>
-      <c r="C75" s="83" t="inlineStr">
+      <c r="C77" s="83" t="inlineStr">
         <is>
           <t>Le fichier n'a pas été débloqué : clic droit ▸ Propriétés ▸ Débloquer.</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="27" customHeight="1">
-      <c r="B76" s="82" t="inlineStr">
+    <row r="78" ht="27" customHeight="1">
+      <c r="B78" s="82" t="inlineStr">
         <is>
           <t>Outlook ne s'ouvre pas</t>
         </is>
       </c>
-      <c r="C76" s="83" t="inlineStr">
+      <c r="C78" s="83" t="inlineStr">
         <is>
           <t>Outlook doit être installé et un profil configuré sur le poste. La version web d'Outlook ne permet pas ce type d'automatisation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="27" customHeight="1">
-      <c r="B77" s="82" t="inlineStr">
-        <is>
-          <t>L'e-mail part sans signature</t>
-        </is>
-      </c>
-      <c r="C77" s="83" t="inlineStr">
-        <is>
-          <t>Laissez la cellule « Signature e-mail » vide dans Paramètres : la signature Outlook par défaut est alors conservée.</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="15" customHeight="1">
-      <c r="B78" s="82" t="inlineStr">
-        <is>
-          <t>Le document Word est vide</t>
-        </is>
-      </c>
-      <c r="C78" s="83" t="inlineStr">
-        <is>
-          <t>Vérifiez le chemin du dossier des modèles dans Paramètres et la présence des fichiers .docx.</t>
         </is>
       </c>
     </row>
     <row r="79" ht="27" customHeight="1">
       <c r="B79" s="82" t="inlineStr">
         <is>
+          <t>L'e-mail part sans signature</t>
+        </is>
+      </c>
+      <c r="C79" s="83" t="inlineStr">
+        <is>
+          <t>Laissez la cellule « Signature e-mail » vide dans Paramètres : la signature Outlook par défaut est alors conservée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="15" customHeight="1">
+      <c r="B80" s="82" t="inlineStr">
+        <is>
+          <t>Le document Word est vide</t>
+        </is>
+      </c>
+      <c r="C80" s="83" t="inlineStr">
+        <is>
+          <t>Vérifiez le chemin du dossier des modèles dans Paramètres et la présence des fichiers .docx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="27" customHeight="1">
+      <c r="B81" s="82" t="inlineStr">
+        <is>
           <t>Une valeur est refusée</t>
         </is>
       </c>
-      <c r="C79" s="83" t="inlineStr">
+      <c r="C81" s="83" t="inlineStr">
         <is>
           <t>Elle ne figure pas dans la liste de l'onglet Paramètres : ajoutez-la, puis cliquez sur « Actualiser les listes ».</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="27" customHeight="1">
-      <c r="B80" s="82" t="inlineStr">
+    <row r="82" ht="27" customHeight="1">
+      <c r="B82" s="82" t="inlineStr">
         <is>
           <t>Le classeur devient lent</t>
         </is>
       </c>
-      <c r="C80" s="83" t="inlineStr">
+      <c r="C82" s="83" t="inlineStr">
         <is>
           <t>Supprimez les lignes vides sous le tableau et archivez les candidatures closes de plus de deux ans (bouton Purge RGPD).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="B55:C55"/>
+  <mergeCells count="15">
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B64:C64"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="B72:C72"/>
     <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B34:C34"/>
     <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="B71:C71"/>
-    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="B65:C65"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>